<commit_message>
feat: finalize phase 4 map panel rollout
Integrate map-note filtering UX, localized content loading, and refreshed city assets/data so phase 4 map panel interactions, translations, and supporting media are versioned together.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/src/data/jeju.xlsx
+++ b/src/data/jeju.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>Title</t>
   </si>
@@ -42,12 +42,6 @@
   </si>
   <si>
     <t>Comment</t>
-  </si>
-  <si>
-    <t>Gangchon Black Pork Seogwipo</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/place/Gangchon+Black+Pork+Seogwipo/data=!4m2!3m1!1s0x350c530de513d08d:0x253aeead1ea9a795</t>
   </si>
   <si>
     <t>Dongmun Traditional Market</t>
@@ -753,11 +747,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1293,7 +1290,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultColWidth="9.55752212389381" defaultRowHeight="13.5" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="40.7787610619469" customWidth="1"/>
@@ -1317,11 +1314,11 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:5">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1405,11 +1402,11 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
-      <c r="A13" t="s">
+    <row r="13" s="1" customFormat="1" spans="1:5">
+      <c r="A13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="2" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1437,15 +1434,10 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
-      <c r="A17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" t="s">
-        <v>36</v>
-      </c>
-    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C13" r:id="rId1" display="https://www.google.com/maps/place/Compose+Coffee/data=!4m2!3m1!1s0x350cfb59b09a1aff:0x345b0e074ce29b20"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>